<commit_message>
update to 2.0_ 250209
</commit_message>
<xml_diff>
--- a/template/IDS_TEMPLATE.xlsx
+++ b/template/IDS_TEMPLATE.xlsx
@@ -1,27 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\c4rlo\OneDrive\Área de Trabalho\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a20ca196396dbff/Documentos/GitHub/ids_converter/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{636DE61C-7C7C-45B9-93A5-6008199F8177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{636DE61C-7C7C-45B9-93A5-6008199F8177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7C095C9-8C9E-4EAA-BE2A-6F4339E1E1AE}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{07C4ADEE-C849-4C6D-8317-4E1D149360FB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{07C4ADEE-C849-4C6D-8317-4E1D149360FB}"/>
   </bookViews>
   <sheets>
-    <sheet name="SPECIFICATIONS" sheetId="5" r:id="rId1"/>
-    <sheet name="APPLICABILITY" sheetId="3" r:id="rId2"/>
-    <sheet name="REQUIREMENTS" sheetId="4" r:id="rId3"/>
-    <sheet name="Support" sheetId="2" r:id="rId4"/>
+    <sheet name="IDS_INFORMATION" sheetId="6" r:id="rId1"/>
+    <sheet name="SPECIFICATIONS" sheetId="5" r:id="rId2"/>
+    <sheet name="APPLICABILITY" sheetId="3" r:id="rId3"/>
+    <sheet name="REQUIREMENTS" sheetId="4" r:id="rId4"/>
+    <sheet name="Support" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">APPLICABILITY!$A$3:$O$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">REQUIREMENTS!$A$3:$K$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SPECIFICATIONS!$A$3:$C$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">APPLICABILITY!$A$3:$O$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">IDS_INFORMATION!$A$3:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">REQUIREMENTS!$A$3:$K$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">SPECIFICATIONS!$A$3:$C$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="240">
   <si>
     <t>specification description</t>
   </si>
@@ -725,6 +727,45 @@
   </si>
   <si>
     <t>prohibited</t>
+  </si>
+  <si>
+    <t>IDS INFORMATION</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Copyright</t>
+  </si>
+  <si>
+    <t>Author (email)</t>
+  </si>
+  <si>
+    <t>IFC Version</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Milestone</t>
+  </si>
+  <si>
+    <t>IDS Version</t>
+  </si>
+  <si>
+    <t>IFC2x3</t>
+  </si>
+  <si>
+    <t>IFC4</t>
+  </si>
+  <si>
+    <t>IFC4x3_ADD2</t>
   </si>
 </sst>
 </file>
@@ -790,7 +831,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -905,6 +946,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="26">
     <border>
@@ -1236,7 +1289,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1449,6 +1502,19 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1764,6 +1830,103 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D746420-E29B-4465-80DC-67484325C9CB}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="33" customHeight="1" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="84.33203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="81" t="s">
+        <v>227</v>
+      </c>
+      <c r="B1" s="81"/>
+    </row>
+    <row r="2" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="81"/>
+      <c r="B2" s="81"/>
+    </row>
+    <row r="3" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="82" t="s">
+        <v>228</v>
+      </c>
+      <c r="B3" s="83"/>
+    </row>
+    <row r="4" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="82" t="s">
+        <v>229</v>
+      </c>
+      <c r="B4" s="83"/>
+    </row>
+    <row r="5" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="82" t="s">
+        <v>236</v>
+      </c>
+      <c r="B5" s="83"/>
+    </row>
+    <row r="6" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="82" t="s">
+        <v>230</v>
+      </c>
+      <c r="B6" s="83"/>
+    </row>
+    <row r="7" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="82" t="s">
+        <v>231</v>
+      </c>
+      <c r="B7" s="83" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="82" t="s">
+        <v>232</v>
+      </c>
+      <c r="B8" s="83"/>
+    </row>
+    <row r="9" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="82" t="s">
+        <v>233</v>
+      </c>
+      <c r="B9" s="83"/>
+    </row>
+    <row r="10" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="82" t="s">
+        <v>234</v>
+      </c>
+      <c r="B10" s="83"/>
+    </row>
+    <row r="11" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="82" t="s">
+        <v>235</v>
+      </c>
+      <c r="B11" s="83"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B2"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{59D16A1C-A058-4439-8070-A8B4317BB649}">
+          <x14:formula1>
+            <xm:f>Support!$F$2:$F$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>B7</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B239F0DE-95D4-4888-9DF4-42CFE324B097}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="33" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -1932,7 +2095,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F52307A5-6B78-4977-A948-3789E427EB48}">
   <dimension ref="A1:O18"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="33" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -2318,7 +2481,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6466653-3344-42ED-8F52-03DB8ECF3CBD}">
   <dimension ref="A1:Q18"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="33" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -2783,7 +2946,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C6BC952-1F10-4032-8D15-0975CA7BBB4C}">
   <dimension ref="A1:F164"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2812,6 +2975,9 @@
       <c r="E1" s="47" t="s">
         <v>22</v>
       </c>
+      <c r="F1" s="84" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -2821,7 +2987,9 @@
       <c r="C2" s="14"/>
       <c r="D2" s="18"/>
       <c r="E2" s="48"/>
-      <c r="F2" s="46"/>
+      <c r="F2" s="85" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
@@ -2839,7 +3007,9 @@
       <c r="E3" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="F3" s="46"/>
+      <c r="F3" s="85" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
@@ -2857,7 +3027,9 @@
       <c r="E4" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="46"/>
+      <c r="F4" s="85" t="s">
+        <v>239</v>
+      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" s="51" t="s">

</xml_diff>